<commit_message>
row 721: name lngt antarctica; karmol and karadeniz names to other names
</commit_message>
<xml_diff>
--- a/batches/2026-09-17_1737ET_fix_other_names_former/lng_carrier_fix.xlsx
+++ b/batches/2026-09-17_1737ET_fix_other_names_former/lng_carrier_fix.xlsx
@@ -511,7 +511,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Rows corrected: 160   Refs checked: 237   Refs dropped/removed: 0</t>
+          <t>Rows corrected: 160   Refs checked: 239   Refs dropped/removed: 0</t>
         </is>
       </c>
     </row>
@@ -20292,14 +20292,14 @@
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr"/>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>Karmol LNGT Powership Antarctica; Northwest Sanderling</t>
+      <c r="G112" s="7" t="inlineStr">
+        <is>
+          <t>Karmol LNGT Powership Antarctica; Karadeniz LNGT Antarctica; Northwest Sanderling</t>
         </is>
       </c>
       <c r="H112" s="6" t="inlineStr">
         <is>
-          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+          <t>https://www.lngindustry.com/regasification/28052025/karpowership-celebrates-fsru-undocking-with-karmol-and-seatrium/, https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr"/>
@@ -29512,7 +29512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F238"/>
+  <dimension ref="A1:F240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -35456,29 +35456,29 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Karmol LNGT Powership Antarctica; Northwest Sanderling</t>
+          <t>Karmol LNGT Powership Antarctica; Karadeniz LNGT Antarctica; Northwest Sanderling</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+          <t>https://www.lngindustry.com/regasification/28052025/karpowership-celebrates-fsru-undocking-with-karmol-and-seatrium/</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Karmol LNGT Powership Antarctica'; the row is renamed 'Karadeniz LNGT Antarctica' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Antarctica (ex-Northwest Sanderling)'</t>
+          <t>former Name 'Karmol LNGT Powership Antarctica' (lngindustry.com, 2025-05-28); the row is renamed 'LNGT Antarctica' by 2026-09-17_1654ET_fix_igu2026_sourced; IGU 2026 prints 'Karadeniz LNGT Antarctica (ex-Northwest Sanderling)' — both IGU names carried here (Baird 2026-09-18)</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>811</t>
+          <t>721</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -35488,7 +35488,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>LNGT Americas; Northwest Stormpetrel</t>
+          <t>Karmol LNGT Powership Antarctica; Karadeniz LNGT Antarctica; Northwest Sanderling</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -35503,14 +35503,14 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>former Name 'LNGT Americas'; the row is renamed 'Karadeniz LNGT Americas' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Americas (ex-Northwest Stormpetrel)'</t>
+          <t>former Name 'Karmol LNGT Powership Antarctica' (lngindustry.com, 2025-05-28); the row is renamed 'LNGT Antarctica' by 2026-09-17_1654ET_fix_igu2026_sourced; IGU 2026 prints 'Karadeniz LNGT Antarctica (ex-Northwest Sanderling)' — both IGU names carried here (Baird 2026-09-18)</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>971</t>
+          <t>721</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -35520,7 +35520,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Puteri Intan</t>
+          <t>Karmol LNGT Powership Antarctica; Karadeniz LNGT Antarctica; Northwest Sanderling</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -35530,19 +35530,19 @@
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Puteri Intan'; the row is renamed 'American Energy' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Karmol LNGT Powership Antarctica' (lngindustry.com, 2025-05-28); the row is renamed 'LNGT Antarctica' by 2026-09-17_1654ET_fix_igu2026_sourced; IGU 2026 prints 'Karadeniz LNGT Antarctica (ex-Northwest Sanderling)' — both IGU names carried here (Baird 2026-09-18)</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>726</t>
+          <t>811</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -35552,7 +35552,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>KLNGTP Black Sea; Portovenere; LNG Portovenere</t>
+          <t>LNGT Americas; Northwest Stormpetrel</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -35562,19 +35562,19 @@
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>former Name 'KLNGTP Black Sea'; the row is renamed 'Karadeniz LNGT Powership Black Sea' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'</t>
+          <t>former Name 'LNGT Americas'; the row is renamed 'Karadeniz LNGT Americas' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Americas (ex-Northwest Stormpetrel)'</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>726</t>
+          <t>971</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -35584,7 +35584,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>KLNGTP Black Sea; Portovenere; LNG Portovenere</t>
+          <t>Puteri Intan</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -35594,19 +35594,19 @@
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>former Name 'KLNGTP Black Sea'; the row is renamed 'Karadeniz LNGT Powership Black Sea' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'</t>
+          <t>former Name 'Puteri Intan'; the row is renamed 'American Energy' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>726</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -35616,7 +35616,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>KLNGTP Marmara; Lerici; LNG Lerici</t>
+          <t>KLNGTP Black Sea; Portovenere; LNG Portovenere</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -35631,14 +35631,14 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>former Name 'KLNGTP Marmara'; the row is renamed 'Karadeniz LNGT Powership Marmara' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'</t>
+          <t>former Name 'KLNGTP Black Sea'; the row is renamed 'Karadeniz LNGT Powership Black Sea' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>727</t>
+          <t>726</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -35648,7 +35648,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>KLNGTP Marmara; Lerici; LNG Lerici</t>
+          <t>KLNGTP Black Sea; Portovenere; LNG Portovenere</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -35658,19 +35658,19 @@
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>former Name 'KLNGTP Marmara'; the row is renamed 'Karadeniz LNGT Powership Marmara' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'</t>
+          <t>former Name 'KLNGTP Black Sea'; the row is renamed 'Karadeniz LNGT Powership Black Sea' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Black Sea (ex-Portovenere / ex-LNG Portovenere)'</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>727</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -35680,29 +35680,29 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Seapeak Hispania</t>
+          <t>KLNGTP Marmara; Lerici; LNG Lerici</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/115017</t>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Seapeak Hispania'; the row is renamed 'Seapeak Jupiter' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'KLNGTP Marmara'; the row is renamed 'Karadeniz LNGT Powership Marmara' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>1004</t>
+          <t>727</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -35712,29 +35712,29 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Seapeak Hispania</t>
+          <t>KLNGTP Marmara; Lerici; LNG Lerici</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/115017</t>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Seapeak Hispania'; the row is renamed 'Seapeak Jupiter' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'KLNGTP Marmara'; the row is renamed 'Karadeniz LNGT Powership Marmara' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'; plus IGU 2026 prints 'Karadeniz LNGT Powership Marmara (ex-Lerici / ex-LNG Lerici)'</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -35744,12 +35744,12 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Energy Frontier</t>
+          <t>Seapeak Hispania</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/116125</t>
+          <t>https://www.shipvault.com/ships/115017</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -35759,14 +35759,14 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Energy Frontier'; the row is renamed 'Arunika Jaya' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Seapeak Hispania'; the row is renamed 'Seapeak Jupiter' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>1004</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -35776,12 +35776,12 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Energy Frontier</t>
+          <t>Seapeak Hispania</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/116125</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/115017</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
@@ -35791,14 +35791,14 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Energy Frontier'; the row is renamed 'Arunika Jaya' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Seapeak Hispania'; the row is renamed 'Seapeak Jupiter' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>562</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -35808,12 +35808,12 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Golar Arctic</t>
+          <t>Energy Frontier</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/116640</t>
+          <t>https://www.shipvault.com/ships/116125</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
@@ -35823,14 +35823,14 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Golar Arctic'; the row is renamed 'SC Serenity' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Energy Frontier'; the row is renamed 'Arunika Jaya' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>562</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -35840,12 +35840,12 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Golar Arctic</t>
+          <t>Energy Frontier</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/116640</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/116125</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -35855,14 +35855,14 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Golar Arctic'; the row is renamed 'SC Serenity' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Energy Frontier'; the row is renamed 'Arunika Jaya' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>866</t>
+          <t>648</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -35872,29 +35872,29 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Metagas Everest</t>
+          <t>Golar Arctic</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+          <t>https://www.shipvault.com/ships/116640</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Metagas Everest'; the row is renamed 'Arctic Metagas' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Golar Arctic'; the row is renamed 'SC Serenity' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>801</t>
+          <t>648</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -35904,29 +35904,29 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>LNG River Orashi</t>
+          <t>Golar Arctic</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/116640</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>former Name 'LNG River Orashi'; the row is renamed 'Gas Garuda' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Golar Arctic'; the row is renamed 'SC Serenity' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>958</t>
+          <t>866</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -35936,7 +35936,7 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>LNG Pioneer; Pioneer Spirit</t>
+          <t>Metagas Everest</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -35951,14 +35951,14 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Pioneer Spirit'; the row is renamed 'Arctic Pioneer' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Metagas Everest'; the row is renamed 'Arctic Metagas' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>459</t>
+          <t>801</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -35968,7 +35968,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Condor LNG; CCH LNG; Methane Lydon Volney</t>
+          <t>LNG River Orashi</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -35983,14 +35983,14 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>former Name 'CCH LNG'; the row is renamed 'LNG Soars' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'LNG Soars (ex-Methane Lydon Volney)'</t>
+          <t>former Name 'LNG River Orashi'; the row is renamed 'Gas Garuda' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>869</t>
+          <t>958</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -36000,7 +36000,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Methane Heather Sally</t>
+          <t>LNG Pioneer; Pioneer Spirit</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -36010,19 +36010,19 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Methane Heather Sally'; the row is renamed 'Shandong Redwood' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Pioneer Spirit'; the row is renamed 'Arctic Pioneer' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>649</t>
+          <t>459</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -36032,7 +36032,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Golar Tundra</t>
+          <t>Condor LNG; CCH LNG; Methane Lydon Volney</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -36047,14 +36047,14 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Golar Tundra'; the row is renamed 'Italis LNG' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'CCH LNG'; the row is renamed 'LNG Soars' by 2026-09-17_1654ET_fix_igu2026_sourced — no ref on hand prints the former name (backend's own published value); held; plus IGU 2026 prints 'LNG Soars (ex-Methane Lydon Volney)'</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>729</t>
+          <t>869</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -36064,29 +36064,29 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Kool Baltic; SCF Melampus</t>
+          <t>Methane Heather Sally</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/3928</t>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Kool Baltic'; the row is renamed 'Cool Baltic' by 2026-09-17_1654ET_fix_igu2026_sourced; plus IGU 2026 prints 'Cool Baltic (ex-SCF Melampus)'</t>
+          <t>former Name 'Methane Heather Sally'; the row is renamed 'Shandong Redwood' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>729</t>
+          <t>649</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -36096,22 +36096,22 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Kool Baltic; SCF Melampus</t>
+          <t>Golar Tundra</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/3928</t>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>former Name 'Kool Baltic'; the row is renamed 'Cool Baltic' by 2026-09-17_1654ET_fix_igu2026_sourced; plus IGU 2026 prints 'Cool Baltic (ex-SCF Melampus)'</t>
+          <t>former Name 'Golar Tundra'; the row is renamed 'Italis LNG' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
@@ -36133,12 +36133,12 @@
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+          <t>https://www.shipvault.com/ships/3928</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
@@ -36150,7 +36150,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>993</t>
+          <t>729</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -36160,29 +36160,29 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>SCF La Perouse</t>
+          <t>Kool Baltic; SCF Melampus</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/3928</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>former Name 'SCF La Perouse'; the row is renamed 'La Perouse' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
+          <t>former Name 'Kool Baltic'; the row is renamed 'Cool Baltic' by 2026-09-17_1654ET_fix_igu2026_sourced; plus IGU 2026 prints 'Cool Baltic (ex-SCF Melampus)'</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>729</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -36192,7 +36192,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Hull 3342 (HDHHI)</t>
+          <t>Kool Baltic; SCF Melampus</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -36207,14 +36207,14 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Apostolos (ex-Hyundai 3342)' — hull-number former name written as the QC §2 placeholder 'Hull 3342 (HDHHI)'</t>
+          <t>former Name 'Kool Baltic'; the row is renamed 'Cool Baltic' by 2026-09-17_1654ET_fix_igu2026_sourced; plus IGU 2026 prints 'Cool Baltic (ex-SCF Melampus)'</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>993</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -36224,7 +36224,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Hull 3341 (HDHHI)</t>
+          <t>SCF La Perouse</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -36239,14 +36239,14 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Assos (ex-3341)' — hull-number former name written as the QC §2 placeholder 'Hull 3341 (HDHHI)'</t>
+          <t>former Name 'SCF La Perouse'; the row is renamed 'La Perouse' by 2026-09-17_1654ET_fix_igu2026_sourced</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>385</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -36256,7 +36256,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Hull 2635 (SHI)</t>
+          <t>Hull 3342 (HDHHI)</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -36271,14 +36271,14 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Athos LNG (ex-Samsung 2635)' — hull-number former name written as the QC §2 placeholder 'Hull 2635 (SHI)'</t>
+          <t>IGU 2026 prints 'Apostolos (ex-Hyundai 3342)' — hull-number former name written as the QC §2 placeholder 'Hull 3342 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>179</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -36288,7 +36288,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Hull 2584 (SHI)</t>
+          <t>Hull 3341 (HDHHI)</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -36303,14 +36303,14 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Celsius Greenwich (ex-2584)' — hull-number former name written as the QC §2 placeholder 'Hull 2584 (SHI)'</t>
+          <t>IGU 2026 prints 'Assos (ex-3341)' — hull-number former name written as the QC §2 placeholder 'Hull 3341 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -36320,7 +36320,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Hull 3293 (HDHHI)</t>
+          <t>Hull 2635 (SHI)</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -36335,14 +36335,14 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Clean Future (ex-3293)' — hull-number former name written as the QC §2 placeholder 'Hull 3293 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Athos LNG (ex-Samsung 2635)' — hull-number former name written as the QC §2 placeholder 'Hull 2635 (SHI)'</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>77</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -36352,7 +36352,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Hull 1881A (Hudong)</t>
+          <t>Hull 2584 (SHI)</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -36362,19 +36362,19 @@
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Greenergy Pearl (ex-Hudong-Zhonghua H1881A)' — hull-number former name written as the QC §2 placeholder 'Hull 1881A (Hudong)'</t>
+          <t>IGU 2026 prints 'Celsius Greenwich (ex-2584)' — hull-number former name written as the QC §2 placeholder 'Hull 2584 (SHI)'</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>173</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -36384,7 +36384,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Hull 1792A (Hudong)</t>
+          <t>Hull 3293 (HDHHI)</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -36399,14 +36399,14 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Hlaitan (ex-H1792A)' — hull-number former name written as the QC §2 placeholder 'Hull 1792A (Hudong)'</t>
+          <t>IGU 2026 prints 'Clean Future (ex-3293)' — hull-number former name written as the QC §2 placeholder 'Hull 3293 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>719</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -36416,7 +36416,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>LNG Unity; Provalys</t>
+          <t>Hull 1881A (Hudong)</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -36431,14 +36431,14 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Karadeniz LNGT Powership Anatolia (ex-LNG Unity / ex-Provalys)'; Provalys</t>
+          <t>IGU 2026 prints 'Greenergy Pearl (ex-Hudong-Zhonghua H1881A)' — hull-number former name written as the QC §2 placeholder 'Hull 1881A (Hudong)'</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>719</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -36448,7 +36448,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>LNG Unity; Provalys</t>
+          <t>Hull 1792A (Hudong)</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -36463,14 +36463,14 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Karadeniz LNGT Powership Anatolia (ex-LNG Unity / ex-Provalys)'; Provalys</t>
+          <t>IGU 2026 prints 'Hlaitan (ex-H1792A)' — hull-number former name written as the QC §2 placeholder 'Hull 1792A (Hudong)'</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>719</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -36480,7 +36480,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Dwiputra</t>
+          <t>LNG Unity; Provalys</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -36490,19 +36490,19 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Karmol LNGT Powership Africa (ex-Dwiputra)'</t>
+          <t>IGU 2026 prints 'Karadeniz LNGT Powership Anatolia (ex-LNG Unity / ex-Provalys)'; Provalys</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>722</t>
+          <t>719</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -36512,7 +36512,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Northwest Shearwater</t>
+          <t>LNG Unity; Provalys</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
@@ -36522,19 +36522,19 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Karmol LNGT Powership Asia (ex-Northwest Shearwater)'</t>
+          <t>IGU 2026 prints 'Karadeniz LNGT Powership Anatolia (ex-LNG Unity / ex-Provalys)'; Provalys</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>720</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -36544,7 +36544,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Hull 1836A (Hudong)</t>
+          <t>Dwiputra</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -36554,19 +36554,19 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Kongtong (ex-Hudong-Zhonghua H1836A)' — hull-number former name written as the QC §2 placeholder 'Hull 1836A (Hudong)'</t>
+          <t>IGU 2026 prints 'Karmol LNGT Powership Africa (ex-Dwiputra)'</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>731</t>
+          <t>722</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -36576,7 +36576,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>SCF Mitre</t>
+          <t>Northwest Shearwater</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -36586,19 +36586,19 @@
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Kool Boreas (ex-SCF Mitre)'</t>
+          <t>IGU 2026 prints 'Karmol LNGT Powership Asia (ex-Northwest Shearwater)'</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>733</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -36608,7 +36608,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>SCF Barents</t>
+          <t>Hull 1836A (Hudong)</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -36623,14 +36623,14 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Kool Firn (ex-SCF Barents)'</t>
+          <t>IGU 2026 prints 'Kongtong (ex-Hudong-Zhonghua H1836A)' — hull-number former name written as the QC §2 placeholder 'Hull 1836A (Hudong)'</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>731</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -36640,7 +36640,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Hull 3221 (HDHHI)</t>
+          <t>SCF Mitre</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -36655,14 +36655,14 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'New Brave (ex-3221)' — hull-number former name written as the QC §2 placeholder 'Hull 3221 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Kool Boreas (ex-SCF Mitre)'</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>733</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -36672,7 +36672,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Hull 3224 (HDHHI)</t>
+          <t>SCF Barents</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -36682,19 +36682,19 @@
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'New Green ST (ex-3224)' — hull-number former name written as the QC §2 placeholder 'Hull 3224 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Kool Firn (ex-SCF Barents)'</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>170</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -36704,7 +36704,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Hull 3222 (HDHHI)</t>
+          <t>Hull 3221 (HDHHI)</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -36719,14 +36719,14 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'New Nature (ex-3222)' — hull-number former name written as the QC §2 placeholder 'Hull 3222 (HDHHI)'</t>
+          <t>IGU 2026 prints 'New Brave (ex-3221)' — hull-number former name written as the QC §2 placeholder 'Hull 3221 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>172</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -36736,7 +36736,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Hull 2592 (SHI)</t>
+          <t>Hull 3224 (HDHHI)</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -36751,14 +36751,14 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Orion Spirit (ex-2592)' — hull-number former name written as the QC §2 placeholder 'Hull 2592 (SHI)'</t>
+          <t>IGU 2026 prints 'New Green ST (ex-3224)' — hull-number former name written as the QC §2 placeholder 'Hull 3224 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>171</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -36768,7 +36768,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Hull 2315 (SHI)</t>
+          <t>Hull 3222 (HDHHI)</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -36778,19 +36778,19 @@
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Pacific Success (ex-Samsung Heavy Industries 2315)' — hull-number former name written as the QC §2 placeholder 'Hull 2315 (SHI)'</t>
+          <t>IGU 2026 prints 'New Nature (ex-3222)' — hull-number former name written as the QC §2 placeholder 'Hull 3222 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -36800,7 +36800,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Hull 3297 (HDHHI)</t>
+          <t>Hull 2592 (SHI)</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -36815,14 +36815,14 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Puteri Ledang (ex-Hull 3297)' — hull-number former name written as the QC §2 placeholder 'Hull 3297 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Orion Spirit (ex-2592)' — hull-number former name written as the QC §2 placeholder 'Hull 2592 (SHI)'</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>177</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -36832,7 +36832,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Hull 3298 (HDHHI)</t>
+          <t>Hull 2315 (SHI)</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -36842,19 +36842,19 @@
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Puteri Mahsuri (ex-Hull 3298)' — hull-number former name written as the QC §2 placeholder 'Hull 3298 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Pacific Success (ex-Samsung Heavy Industries 2315)' — hull-number former name written as the QC §2 placeholder 'Hull 2315 (SHI)'</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>176</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -36864,7 +36864,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Hull 3295 (HDHHI)</t>
+          <t>Hull 3297 (HDHHI)</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -36879,14 +36879,14 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Puteri Santubong (ex-Hull 3295)' — hull-number former name written as the QC §2 placeholder 'Hull 3295 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Puteri Ledang (ex-Hull 3297)' — hull-number former name written as the QC §2 placeholder 'Hull 3297 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>972</t>
+          <t>177</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -36896,7 +36896,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Hull 3299 (HSHI)</t>
+          <t>Hull 3298 (HDHHI)</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -36911,14 +36911,14 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Puteri Mayang (ex-Hull 3299)' — hull-number former name written as the QC §2 placeholder 'Hull 3299 (HSHI)'</t>
+          <t>IGU 2026 prints 'Puteri Mahsuri (ex-Hull 3298)' — hull-number former name written as the QC §2 placeholder 'Hull 3298 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>174</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -36928,7 +36928,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Hull H1793A (Hudong)</t>
+          <t>Hull 3295 (HDHHI)</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -36938,19 +36938,19 @@
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Limail (ex-Hudong Hull 1793A)' — hull-number former name written as the QC §2 placeholder 'Hull H1793A (Hudong)'</t>
+          <t>IGU 2026 prints 'Puteri Santubong (ex-Hull 3295)' — hull-number former name written as the QC §2 placeholder 'Hull 3295 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>885</t>
+          <t>972</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -36960,7 +36960,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Hull 2527 (Hanwha)</t>
+          <t>Hull 3299 (HSHI)</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -36975,14 +36975,14 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'MOL Azure (ex-Hull 2527)' — hull-number former name written as the QC §2 placeholder 'Hull 2527 (Hanwha)'</t>
+          <t>IGU 2026 prints 'Puteri Mayang (ex-Hull 3299)' — hull-number former name written as the QC §2 placeholder 'Hull 3299 (HSHI)'</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>915</t>
+          <t>257</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -36992,7 +36992,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Hull 3225 (HDHHI)</t>
+          <t>Hull H1793A (Hudong)</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -37002,19 +37002,19 @@
       </c>
       <c r="E234" s="2" t="inlineStr">
         <is>
-          <t>PASS (corroborates)</t>
+          <t>PASS (OK (all tokens present))</t>
         </is>
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'New Oasis (ex-Hyundai 3225)' — hull-number former name written as the QC §2 placeholder 'Hull 3225 (HDHHI)'</t>
+          <t>IGU 2026 prints 'Limail (ex-Hudong Hull 1793A)' — hull-number former name written as the QC §2 placeholder 'Hull H1793A (Hudong)'</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>885</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -37024,7 +37024,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Hull 2566 (Hanwha)</t>
+          <t>Hull 2527 (Hanwha)</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -37039,14 +37039,14 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Esteem Fuji (ex-Hull 2566)' — hull-number former name written as the QC §2 placeholder 'Hull 2566 (Hanwha)'</t>
+          <t>IGU 2026 prints 'MOL Azure (ex-Hull 2527)' — hull-number former name written as the QC §2 placeholder 'Hull 2527 (Hanwha)'</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>915</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -37056,7 +37056,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Hull 2537 (Hanwha)</t>
+          <t>Hull 3225 (HDHHI)</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -37071,14 +37071,14 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Maran Gas Syros (ex-ABCDE (2537))' — hull-number former name written as the QC §2 placeholder 'Hull 2537 (Hanwha)'</t>
+          <t>IGU 2026 prints 'New Oasis (ex-Hyundai 3225)' — hull-number former name written as the QC §2 placeholder 'Hull 3225 (HDHHI)'</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>59</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -37088,7 +37088,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Hull H1892A (Hudong)</t>
+          <t>Hull 2566 (Hanwha)</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -37098,42 +37098,106 @@
       </c>
       <c r="E237" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (all tokens present))</t>
+          <t>PASS (corroborates)</t>
         </is>
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>IGU 2026 prints 'Ocean Inspiration (ex-Hudong-Zhonghua H1892A)' — hull-number former name written as the QC §2 placeholder 'Hull H1892A (Hudong)'</t>
+          <t>IGU 2026 prints 'Esteem Fuji (ex-Hull 2566)' — hull-number former name written as the QC §2 placeholder 'Hull 2566 (Hanwha)'</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Other names</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>Hull 2537 (Hanwha)</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>PASS (corroborates)</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>IGU 2026 prints 'Maran Gas Syros (ex-ABCDE (2537))' — hull-number former name written as the QC §2 placeholder 'Hull 2537 (Hanwha)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Other names</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>Hull H1892A (Hudong)</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (all tokens present))</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>IGU 2026 prints 'Ocean Inspiration (ex-Hudong-Zhonghua H1892A)' — hull-number former name written as the QC §2 placeholder 'Hull H1892A (Hudong)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
           <t>1111</t>
         </is>
       </c>
-      <c r="B238" s="2" t="inlineStr">
+      <c r="B240" s="2" t="inlineStr">
         <is>
           <t>Other names</t>
         </is>
       </c>
-      <c r="C238" s="2" t="inlineStr">
+      <c r="C240" s="2" t="inlineStr">
         <is>
           <t>Hull 2535 (Hanwha)</t>
         </is>
       </c>
-      <c r="D238" s="2" t="inlineStr">
+      <c r="D240" s="2" t="inlineStr">
         <is>
           <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
-      <c r="E238" s="2" t="inlineStr">
+      <c r="E240" s="2" t="inlineStr">
         <is>
           <t>PASS (corroborates)</t>
         </is>
       </c>
-      <c r="F238" s="2" t="inlineStr">
+      <c r="F240" s="2" t="inlineStr">
         <is>
           <t>IGU 2026 prints 'Woodside Barrumbara (ex-2535)' — hull-number former name written as the QC §2 placeholder 'Hull 2535 (Hanwha)'</t>
         </is>

</xml_diff>